<commit_message>
Add live Partiful sync and dynamic agenda planning
Add logistics-aware agenda recalculation with preference defaults, local agenda run persistence, and schedule readback support.

Add browser, headless, and Twilio-backed Partiful sync helpers with Deno tasks and regression tests.

Regenerate Tech Week route artifacts against the exact 15 Cliff Street home anchor.
</commit_message>
<xml_diff>
--- a/outputs/accolades/techweek_nyc_accolades_detailed_calendar.xlsx
+++ b/outputs/accolades/techweek_nyc_accolades_detailed_calendar.xlsx
@@ -105,7 +105,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-01 13:22</t>
+          <t xml:space="preserve">2026-06-01 13:21</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -120,7 +120,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FiDi home base -&gt; Flatiron</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038 -&gt; Flatiron</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -140,12 +140,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">38</t>
+          <t xml:space="preserve">39</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Wall St (2/3); subway 31 min; walk 2 min from 23 St-Baruch College (4/6); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 3 min to Fulton St (2/3); subway 29 min; walk 2 min from 23 St-Baruch College (4/6); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -684,27 +684,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-01 21:35</t>
+          <t xml:space="preserve">2026-06-01 21:30</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel back to FiDi</t>
+          <t xml:space="preserve">Travel home</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Source Must Win -&gt; FiDi home base</t>
+          <t xml:space="preserve">Open Source Must Win -&gt; 15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">approx_fidi_anchor</t>
+          <t xml:space="preserve">exact_home_base</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wall St, New York, NY</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">35</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk approx 35 min / 2751 m using OSM-geocoded points.</t>
+          <t xml:space="preserve">Walk approx 30 min / 2327 m using OSM-geocoded points.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-02 11:13</t>
+          <t xml:space="preserve">2026-06-02 11:12</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">FiDi home base -&gt; Midtown</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038 -&gt; Midtown</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">47</t>
+          <t xml:space="preserve">48</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Wall St (2/3); subway 40 min; walk 2 min from 42 St-Bryant Pk (B/D/F/M); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 3 min to Fulton St (2/3); subway 38 min; walk 2 min from 42 St-Bryant Pk (B/D/F/M); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1422,27 +1422,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-02 21:20</t>
+          <t xml:space="preserve">2026-06-02 21:21</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel back to FiDi</t>
+          <t xml:space="preserve">Travel home</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Future of DevEx -&gt; FiDi home base</t>
+          <t xml:space="preserve">Future of DevEx -&gt; 15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">approx_fidi_anchor</t>
+          <t xml:space="preserve">exact_home_base</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wall St, New York, NY</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1452,12 +1452,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Prince St (N/Q/R/W); subway 15 min; walk 0 min from Wall St (2/3); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 0 min to Prince St (N/Q/R/W); subway 13 min; walk 3 min from Fulton St (2/3); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-03 11:29</t>
+          <t xml:space="preserve">2026-06-03 11:28</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">FiDi home base -&gt; Chelsea</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038 -&gt; Chelsea</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">31</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Wall St (2/3); subway 22 min; walk 4 min from 23 St (A/C/E); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 3 min to Fulton St (2/3); subway 20 min; walk 4 min from 23 St (A/C/E); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2570,27 +2570,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-03 20:50</t>
+          <t xml:space="preserve">2026-06-03 20:51</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel back to FiDi</t>
+          <t xml:space="preserve">Travel home</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP in the Wild: Panel &amp; Night of Networking -&gt; FiDi home base</t>
+          <t xml:space="preserve">MCP in the Wild: Panel &amp; Night of Networking -&gt; 15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">approx_fidi_anchor</t>
+          <t xml:space="preserve">exact_home_base</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wall St, New York, NY</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2600,12 +2600,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 1 min to Astor Pl (4/6); subway 14 min; walk 0 min from Wall St (2/3); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 1 min to Astor Pl (4/6); subway 12 min; walk 3 min from Fulton St (2/3); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-04 15:36</t>
+          <t xml:space="preserve">2026-06-04 15:35</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">FiDi home base -&gt; SoHo</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038 -&gt; SoHo</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2682,12 +2682,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Wall St (2/3); subway 19 min; walk 0 min from Prince St (N/Q/R/W); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 3 min to Fulton St (2/3); subway 17 min; walk 0 min from Prince St (N/Q/R/W); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3144,27 +3144,27 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-04 19:20</t>
+          <t xml:space="preserve">2026-06-04 19:21</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel back to FiDi</t>
+          <t xml:space="preserve">Travel home</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shipping Faster with AI Coding Agents: What's Working and What's Not -&gt; FiDi home base</t>
+          <t xml:space="preserve">Shipping Faster with AI Coding Agents: What's Working and What's Not -&gt; 15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">approx_fidi_anchor</t>
+          <t xml:space="preserve">exact_home_base</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wall St, New York, NY</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3174,12 +3174,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t xml:space="preserve">21</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Prince St (N/Q/R/W); subway 15 min; walk 0 min from Wall St (2/3); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 0 min to Prince St (N/Q/R/W); subway 13 min; walk 3 min from Fulton St (2/3); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-05 16:22</t>
+          <t xml:space="preserve">2026-06-05 16:21</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">FiDi home base -&gt; Union Square</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038 -&gt; Union Square</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3338,12 +3338,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t xml:space="preserve">38</t>
+          <t xml:space="preserve">39</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 0 min to Wall St (2/3); subway 29 min; walk 4 min from 14 St-Union Sq (N/Q/R/W); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 3 min to Fulton St (2/3); subway 27 min; walk 4 min from 14 St-Union Sq (N/Q/R/W); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3554,27 +3554,27 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-05 20:22</t>
+          <t xml:space="preserve">2026-06-05 20:23</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel back to FiDi</t>
+          <t xml:space="preserve">Travel home</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bare Metal Happy Hour: Autonomous Systems &amp; Agent Fleet Orchestration -&gt; FiDi home base</t>
+          <t xml:space="preserve">Bare Metal Happy Hour: Autonomous Systems &amp; Agent Fleet Orchestration -&gt; 15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">approx_fidi_anchor</t>
+          <t xml:space="preserve">exact_home_base</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wall St, New York, NY</t>
+          <t xml:space="preserve">15 Cliff Street, New York, NY 10038</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3584,12 +3584,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t xml:space="preserve">22</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk 4 min to 14 St-Union Sq (N/Q/R/W); subway 13 min; walk 0 min from Wall St (2/3); includes 5 min buffer.</t>
+          <t xml:space="preserve">Walk 4 min to 14 St-Union Sq (N/Q/R/W); subway 11 min; walk 3 min from Fulton St (2/3); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">

</xml_diff>